<commit_message>
Align Task List with ECOSYSTEM.md suite contract
Bring sample columns, landing/help copy, and docs in line with the
Website ecosystem contract: PM starter fields only, prefer End Date,
Duration/Tooltips as later-supported, and ship ECOSYSTEM.md locally.
Bump to 1.0.3.0 and refresh branded/whitelabel packages + website-sync.

Co-authored-by: JonasL <Prez0@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/taskList/downloads/TaskListSampleData.xlsx
+++ b/taskList/downloads/TaskListSampleData.xlsx
@@ -7,19 +7,24 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Projects" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Start here" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Projects" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Projects'!$A$1:$G$6</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="0&quot;%&quot;"/>
+    <numFmt numFmtId="166" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,16 +32,109 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="22"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000F3D36"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000F3D36"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A6B5C"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="003D5A54"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001A6B5C"/>
+      <sz val="11"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001B7F5A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00B86E00"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00B42318"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F3D36"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F2EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A6B5C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3FAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D8F3E7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCEFC7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F9D8D5"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -44,13 +142,54 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C5D9D2"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C5D9D2"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C5D9D2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C5D9D2"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,417 +552,308 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="000F3D36"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="82" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DataLund Task List</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Core project columns only — swap in your own rows</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="n"/>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Quick start</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>1. Import taskList.pbiviz</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>2. Load Projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>3. Bind Project, RAG, Group, Project lead, Progress, Start Date, End Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Project = Task well · Project lead = Resource well. Full suite → DatalundSuiteSample.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>https://datalund.no/visuals/task-list/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002DD4BF"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>RAG</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Phase</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>Project lead</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>Progress</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Start date</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Estimated end</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Next milestone</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Obstacles</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>End Date</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>North Sea Hub</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>Green</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="10" t="inlineStr">
         <is>
           <t>Delivery</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="10" t="inlineStr">
         <is>
           <t>Ada Ng</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="12" t="n">
         <v>72</v>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="F2" s="13" t="n">
         <v>46184</v>
       </c>
-      <c r="G2" s="1" t="n">
+      <c r="G2" s="13" t="n">
         <v>46284</v>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>FAT complete</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>On track for Q3</t>
-        </is>
-      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Arctic Link</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Amber</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="14" t="inlineStr">
         <is>
           <t>Delivery</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="14" t="inlineStr">
         <is>
           <t>Bo Berg</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="16" t="n">
         <v>45</v>
       </c>
-      <c r="F3" s="1" t="n">
+      <c r="F3" s="17" t="n">
         <v>46154</v>
       </c>
-      <c r="G3" s="1" t="n">
+      <c r="G3" s="17" t="n">
         <v>46264</v>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Cable pull</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Weather window</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Watch supplier lead time</t>
-        </is>
-      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Yard Retrofit</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>Initiation</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>Cara Diaz</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="12" t="n">
         <v>18</v>
       </c>
-      <c r="F4" s="1" t="n">
+      <c r="F4" s="13" t="n">
         <v>46214</v>
       </c>
-      <c r="G4" s="1" t="n">
+      <c r="G4" s="13" t="n">
         <v>46254</v>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Scope freeze</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Budget overrun</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Critical path slip</t>
-        </is>
-      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Digital Twin v2</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>On track</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>Build</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="14" t="inlineStr">
         <is>
           <t>Dan Okonkwo</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="16" t="n">
         <v>88</v>
       </c>
-      <c r="F5" s="1" t="n">
+      <c r="F5" s="17" t="n">
         <v>46124</v>
       </c>
-      <c r="G5" s="1" t="n">
+      <c r="G5" s="17" t="n">
         <v>46259</v>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>UAT</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>HSEQ Pulse</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>At risk</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Operate</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Eva Holm</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>55</v>
-      </c>
-      <c r="F6" s="1" t="n">
-        <v>46044</v>
-      </c>
-      <c r="G6" s="1" t="n">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Port Expansion</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Amber</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>Finn Olsen</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="F6" s="13" t="n">
         <v>46249</v>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Audit prep</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Missing evidence</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Port Expansion</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Plan</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Finn Olsen</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>12</v>
-      </c>
-      <c r="F7" s="1" t="n">
-        <v>46249</v>
-      </c>
-      <c r="G7" s="1" t="n">
+      <c r="G6" s="13" t="n">
         <v>46424</v>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Permits</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Crew Roster</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Operate</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Ada Ng</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>100</v>
-      </c>
-      <c r="F8" s="1" t="n">
-        <v>45844</v>
-      </c>
-      <c r="G8" s="1" t="n">
-        <v>46234</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Spare Parts AI</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Yellow</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Bo Berg</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>33</v>
-      </c>
-      <c r="F9" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="G9" s="1" t="n">
-        <v>46334</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Model v1</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Data quality</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Align Task List with ECOSYSTEM.md suite contract (#5)
Bring sample columns, landing/help copy, and docs in line with the
Website ecosystem contract: PM starter fields only, prefer End Date,
Duration/Tooltips as later-supported, and ship ECOSYSTEM.md locally.
Bump to 1.0.3.0 and refresh branded/whitelabel packages + website-sync.

Co-authored-by: Cursor Agent <cursoragent@cursor.com>
Co-authored-by: JonasL <Prez0@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/taskList/downloads/TaskListSampleData.xlsx
+++ b/taskList/downloads/TaskListSampleData.xlsx
@@ -7,19 +7,24 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Projects" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Start here" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Projects" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Projects'!$A$1:$G$6</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="0&quot;%&quot;"/>
+    <numFmt numFmtId="166" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,16 +32,109 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="22"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000F3D36"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000F3D36"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A6B5C"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="003D5A54"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001A6B5C"/>
+      <sz val="11"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001B7F5A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00B86E00"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00B42318"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F3D36"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F2EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A6B5C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3FAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D8F3E7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCEFC7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F9D8D5"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -44,13 +142,54 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C5D9D2"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C5D9D2"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C5D9D2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C5D9D2"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,417 +552,308 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="000F3D36"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="82" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DataLund Task List</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Core project columns only — swap in your own rows</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="n"/>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Quick start</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>1. Import taskList.pbiviz</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>2. Load Projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>3. Bind Project, RAG, Group, Project lead, Progress, Start Date, End Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Project = Task well · Project lead = Resource well. Full suite → DatalundSuiteSample.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>https://datalund.no/visuals/task-list/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002DD4BF"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>RAG</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Phase</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>Project lead</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>Progress</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Start date</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Estimated end</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Next milestone</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Obstacles</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>End Date</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>North Sea Hub</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>Green</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="10" t="inlineStr">
         <is>
           <t>Delivery</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="10" t="inlineStr">
         <is>
           <t>Ada Ng</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="12" t="n">
         <v>72</v>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="F2" s="13" t="n">
         <v>46184</v>
       </c>
-      <c r="G2" s="1" t="n">
+      <c r="G2" s="13" t="n">
         <v>46284</v>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>FAT complete</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>On track for Q3</t>
-        </is>
-      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Arctic Link</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Amber</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="14" t="inlineStr">
         <is>
           <t>Delivery</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="14" t="inlineStr">
         <is>
           <t>Bo Berg</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="16" t="n">
         <v>45</v>
       </c>
-      <c r="F3" s="1" t="n">
+      <c r="F3" s="17" t="n">
         <v>46154</v>
       </c>
-      <c r="G3" s="1" t="n">
+      <c r="G3" s="17" t="n">
         <v>46264</v>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Cable pull</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Weather window</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Watch supplier lead time</t>
-        </is>
-      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Yard Retrofit</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>Initiation</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>Cara Diaz</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="12" t="n">
         <v>18</v>
       </c>
-      <c r="F4" s="1" t="n">
+      <c r="F4" s="13" t="n">
         <v>46214</v>
       </c>
-      <c r="G4" s="1" t="n">
+      <c r="G4" s="13" t="n">
         <v>46254</v>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Scope freeze</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Budget overrun</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Critical path slip</t>
-        </is>
-      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Digital Twin v2</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>On track</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>Build</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="14" t="inlineStr">
         <is>
           <t>Dan Okonkwo</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="16" t="n">
         <v>88</v>
       </c>
-      <c r="F5" s="1" t="n">
+      <c r="F5" s="17" t="n">
         <v>46124</v>
       </c>
-      <c r="G5" s="1" t="n">
+      <c r="G5" s="17" t="n">
         <v>46259</v>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>UAT</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>HSEQ Pulse</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>At risk</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Operate</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Eva Holm</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>55</v>
-      </c>
-      <c r="F6" s="1" t="n">
-        <v>46044</v>
-      </c>
-      <c r="G6" s="1" t="n">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Port Expansion</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Amber</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>Finn Olsen</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="F6" s="13" t="n">
         <v>46249</v>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Audit prep</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Missing evidence</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Port Expansion</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Plan</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Finn Olsen</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>12</v>
-      </c>
-      <c r="F7" s="1" t="n">
-        <v>46249</v>
-      </c>
-      <c r="G7" s="1" t="n">
+      <c r="G6" s="13" t="n">
         <v>46424</v>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Permits</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Crew Roster</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Operate</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Ada Ng</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>100</v>
-      </c>
-      <c r="F8" s="1" t="n">
-        <v>45844</v>
-      </c>
-      <c r="G8" s="1" t="n">
-        <v>46234</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Spare Parts AI</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Yellow</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Bo Berg</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>33</v>
-      </c>
-      <c r="F9" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="G9" s="1" t="n">
-        <v>46334</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Model v1</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Data quality</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>